<commit_message>
[Update] Monster, MonsterCondition, MonsterAnimation, 맵 NavMesh 추가 및 베이크
</commit_message>
<xml_diff>
--- a/Assets/Resources/Excels/MonsterSheets.xlsx
+++ b/Assets/Resources/Excels/MonsterSheets.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Project\In_You\Assets\Resources\Excels\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FC19EBC5-8725-41DE-9ADD-3BAE8284844D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B6689E56-16D5-46FE-BBB0-6E0070C22C5C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{370970DB-CFD6-4742-B8DB-B40C1E5D66D6}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="21">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="19">
   <si>
     <t>id</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -49,14 +49,6 @@
   </si>
   <si>
     <t>iconPath</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>colliderRadius</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>colliderHeight</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
@@ -481,7 +473,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{02DBBB59-976D-468B-AEDF-09065DDEF90E}">
-  <dimension ref="A1:O7"/>
+  <dimension ref="A1:M7"/>
   <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="11.75" customWidth="1"/>
@@ -499,7 +491,7 @@
     <col min="14" max="14" width="8.75" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -507,7 +499,7 @@
         <v>1</v>
       </c>
       <c r="C1" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="D1" t="s">
         <v>2</v>
@@ -539,77 +531,71 @@
       <c r="M1" t="s">
         <v>11</v>
       </c>
-      <c r="N1" t="s">
-        <v>12</v>
-      </c>
-      <c r="O1" t="s">
-        <v>13</v>
-      </c>
     </row>
-    <row r="2" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A2">
         <v>10001</v>
       </c>
       <c r="B2" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="C2" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
     </row>
-    <row r="3" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A3">
         <v>10002</v>
       </c>
       <c r="B3" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="C3" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
     </row>
-    <row r="4" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A4">
         <v>10003</v>
       </c>
       <c r="B4" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="C4" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
     </row>
-    <row r="5" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A5">
         <v>10004</v>
       </c>
       <c r="B5" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="C5" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
     </row>
-    <row r="6" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A6">
         <v>10005</v>
       </c>
       <c r="B6" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="C6" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
     </row>
-    <row r="7" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A7">
         <v>10006</v>
       </c>
       <c r="B7" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="C7" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
[Update] MonsterSpawner 1차 완료
</commit_message>
<xml_diff>
--- a/Assets/Resources/Excels/MonsterSheets.xlsx
+++ b/Assets/Resources/Excels/MonsterSheets.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Project\In_You\Assets\Resources\Excels\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B6689E56-16D5-46FE-BBB0-6E0070C22C5C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E941ED18-5740-4DEA-9F3D-7A189908179E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{370970DB-CFD6-4742-B8DB-B40C1E5D66D6}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="19">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="19">
   <si>
     <t>id</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -64,30 +64,10 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>chasePeriod</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>attackDamage</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>attackPeriod</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>duration</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>waitTime</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>Bug</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>description</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
@@ -110,6 +90,22 @@
   <si>
     <t>Raven</t>
     <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>/Prefabs/Monster/Raven</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>/Prefabs/Monster/Spider</t>
+  </si>
+  <si>
+    <t>/Prefabs/Monster/RedZombie</t>
+  </si>
+  <si>
+    <t>/Prefabs/Monster/PurpleZombie</t>
+  </si>
+  <si>
+    <t>/Prefabs/Monster/CrawlZombie</t>
   </si>
 </sst>
 </file>
@@ -473,7 +469,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{02DBBB59-976D-468B-AEDF-09065DDEF90E}">
-  <dimension ref="A1:M7"/>
+  <dimension ref="A1:I6"/>
   <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="11.75" customWidth="1"/>
@@ -482,8 +478,8 @@
     <col min="5" max="5" width="31.375" customWidth="1"/>
     <col min="6" max="6" width="13.75" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="12.625" customWidth="1"/>
-    <col min="8" max="8" width="7.5" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="11.5" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="14.5" customWidth="1"/>
+    <col min="9" max="9" width="13.25" customWidth="1"/>
     <col min="10" max="10" width="14.625" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="11.875" bestFit="1" customWidth="1"/>
     <col min="12" max="12" width="14.125" bestFit="1" customWidth="1"/>
@@ -491,7 +487,7 @@
     <col min="14" max="14" width="8.75" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -499,7 +495,7 @@
         <v>1</v>
       </c>
       <c r="C1" t="s">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="D1" t="s">
         <v>2</v>
@@ -519,83 +515,135 @@
       <c r="I1" t="s">
         <v>7</v>
       </c>
-      <c r="J1" t="s">
-        <v>8</v>
-      </c>
-      <c r="K1" t="s">
-        <v>9</v>
-      </c>
-      <c r="L1" t="s">
-        <v>10</v>
-      </c>
-      <c r="M1" t="s">
-        <v>11</v>
-      </c>
     </row>
-    <row r="2" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A2">
         <v>10001</v>
       </c>
       <c r="B2" t="s">
+        <v>13</v>
+      </c>
+      <c r="C2" t="s">
+        <v>13</v>
+      </c>
+      <c r="D2" t="s">
+        <v>14</v>
+      </c>
+      <c r="F2">
+        <v>5</v>
+      </c>
+      <c r="G2">
+        <v>1.1000000000000001</v>
+      </c>
+      <c r="H2">
+        <v>1</v>
+      </c>
+      <c r="I2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A3">
+        <v>10003</v>
+      </c>
+      <c r="B3" t="s">
+        <v>9</v>
+      </c>
+      <c r="C3" t="s">
+        <v>9</v>
+      </c>
+      <c r="D3" t="s">
+        <v>15</v>
+      </c>
+      <c r="F3">
+        <v>5</v>
+      </c>
+      <c r="G3">
+        <v>0.8</v>
+      </c>
+      <c r="H3">
+        <v>1</v>
+      </c>
+      <c r="I3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A4">
+        <v>10004</v>
+      </c>
+      <c r="B4" t="s">
+        <v>10</v>
+      </c>
+      <c r="C4" t="s">
+        <v>10</v>
+      </c>
+      <c r="D4" t="s">
+        <v>16</v>
+      </c>
+      <c r="F4">
+        <v>5</v>
+      </c>
+      <c r="G4">
+        <v>1</v>
+      </c>
+      <c r="H4">
+        <v>1</v>
+      </c>
+      <c r="I4">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A5">
+        <v>10005</v>
+      </c>
+      <c r="B5" t="s">
+        <v>11</v>
+      </c>
+      <c r="C5" t="s">
+        <v>11</v>
+      </c>
+      <c r="D5" t="s">
+        <v>17</v>
+      </c>
+      <c r="F5">
+        <v>5</v>
+      </c>
+      <c r="G5">
+        <v>1</v>
+      </c>
+      <c r="H5">
+        <v>1</v>
+      </c>
+      <c r="I5">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A6">
+        <v>10006</v>
+      </c>
+      <c r="B6" t="s">
+        <v>12</v>
+      </c>
+      <c r="C6" t="s">
+        <v>12</v>
+      </c>
+      <c r="D6" t="s">
         <v>18</v>
       </c>
-      <c r="C2" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="3" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A3">
-        <v>10002</v>
-      </c>
-      <c r="B3" t="s">
-        <v>12</v>
-      </c>
-      <c r="C3" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="4" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A4">
-        <v>10003</v>
-      </c>
-      <c r="B4" t="s">
-        <v>14</v>
-      </c>
-      <c r="C4" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="5" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A5">
-        <v>10004</v>
-      </c>
-      <c r="B5" t="s">
-        <v>15</v>
-      </c>
-      <c r="C5" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="6" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A6">
-        <v>10005</v>
-      </c>
-      <c r="B6" t="s">
-        <v>16</v>
-      </c>
-      <c r="C6" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="7" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A7">
-        <v>10006</v>
-      </c>
-      <c r="B7" t="s">
-        <v>17</v>
-      </c>
-      <c r="C7" t="s">
-        <v>17</v>
+      <c r="F6">
+        <v>5</v>
+      </c>
+      <c r="G6">
+        <v>0.7</v>
+      </c>
+      <c r="H6">
+        <v>1</v>
+      </c>
+      <c r="I6">
+        <v>1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
[Update] MonsterAnimation 업데이트, 버그 수정
</commit_message>
<xml_diff>
--- a/Assets/Resources/Excels/MonsterSheets.xlsx
+++ b/Assets/Resources/Excels/MonsterSheets.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Project\In_You\Assets\Resources\Excels\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E941ED18-5740-4DEA-9F3D-7A189908179E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{43F84C8C-F9B4-4635-AF6C-E1D7FBFBF8B8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{370970DB-CFD6-4742-B8DB-B40C1E5D66D6}"/>
   </bookViews>
@@ -34,78 +34,74 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="19">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="23" uniqueCount="18">
+  <si>
+    <t>displayTitle</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>prefabPath</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>maxHp</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>moveSpeed</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>attractDistance</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>attackDamage</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>description</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Spider</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>RedZombie</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>PurpleZombie</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>CrawlZombie</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Raven</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>/Prefabs/Monster/Raven</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>/Prefabs/Monster/Spider</t>
+  </si>
+  <si>
+    <t>/Prefabs/Monster/RedZombie</t>
+  </si>
+  <si>
+    <t>/Prefabs/Monster/PurpleZombie</t>
+  </si>
+  <si>
+    <t>/Prefabs/Monster/CrawlZombie</t>
+  </si>
   <si>
     <t>id</t>
     <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>displayTitle</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>prefabPath</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>iconPath</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>maxHp</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>moveSpeed</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>attractDistance</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>attackDamage</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>description</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>Spider</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>RedZombie</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>PurpleZombie</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>CrawlZombie</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>Raven</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>/Prefabs/Monster/Raven</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>/Prefabs/Monster/Spider</t>
-  </si>
-  <si>
-    <t>/Prefabs/Monster/RedZombie</t>
-  </si>
-  <si>
-    <t>/Prefabs/Monster/PurpleZombie</t>
-  </si>
-  <si>
-    <t>/Prefabs/Monster/CrawlZombie</t>
   </si>
 </sst>
 </file>
@@ -469,9 +465,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{02DBBB59-976D-468B-AEDF-09065DDEF90E}">
-  <dimension ref="A1:I6"/>
+  <dimension ref="A1:H6"/>
   <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
   <cols>
+    <col min="1" max="1" width="10.25" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="11.75" customWidth="1"/>
     <col min="3" max="3" width="13.125" customWidth="1"/>
     <col min="4" max="4" width="33.125" customWidth="1"/>
@@ -487,162 +484,159 @@
     <col min="14" max="14" width="8.75" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
+        <v>17</v>
+      </c>
+      <c r="B1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
-        <v>1</v>
-      </c>
       <c r="C1" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="D1" t="s">
+        <v>1</v>
+      </c>
+      <c r="E1" t="s">
         <v>2</v>
       </c>
-      <c r="E1" t="s">
+      <c r="F1" t="s">
         <v>3</v>
       </c>
-      <c r="F1" t="s">
+      <c r="G1" t="s">
         <v>4</v>
       </c>
-      <c r="G1" t="s">
+      <c r="H1" t="s">
         <v>5</v>
       </c>
-      <c r="H1" t="s">
-        <v>6</v>
-      </c>
-      <c r="I1" t="s">
-        <v>7</v>
-      </c>
     </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A2">
         <v>10001</v>
       </c>
       <c r="B2" t="s">
+        <v>11</v>
+      </c>
+      <c r="C2" t="s">
+        <v>11</v>
+      </c>
+      <c r="D2" t="s">
+        <v>12</v>
+      </c>
+      <c r="E2">
+        <v>5</v>
+      </c>
+      <c r="F2">
+        <v>1.1000000000000001</v>
+      </c>
+      <c r="G2">
+        <v>1</v>
+      </c>
+      <c r="H2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A3">
+        <v>10002</v>
+      </c>
+      <c r="B3" t="s">
+        <v>7</v>
+      </c>
+      <c r="C3" t="s">
+        <v>7</v>
+      </c>
+      <c r="D3" t="s">
         <v>13</v>
       </c>
-      <c r="C2" t="s">
-        <v>13</v>
-      </c>
-      <c r="D2" t="s">
+      <c r="E3">
+        <v>5</v>
+      </c>
+      <c r="F3">
+        <v>0.8</v>
+      </c>
+      <c r="G3">
+        <v>1</v>
+      </c>
+      <c r="H3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A4">
+        <v>10003</v>
+      </c>
+      <c r="B4" t="s">
+        <v>8</v>
+      </c>
+      <c r="C4" t="s">
+        <v>8</v>
+      </c>
+      <c r="D4" t="s">
         <v>14</v>
       </c>
-      <c r="F2">
+      <c r="E4">
         <v>5</v>
       </c>
-      <c r="G2">
-        <v>1.1000000000000001</v>
-      </c>
-      <c r="H2">
-        <v>1</v>
-      </c>
-      <c r="I2">
+      <c r="F4">
+        <v>1</v>
+      </c>
+      <c r="G4">
+        <v>1</v>
+      </c>
+      <c r="H4">
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A3">
-        <v>10003</v>
-      </c>
-      <c r="B3" t="s">
+    <row r="5" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A5">
+        <v>10004</v>
+      </c>
+      <c r="B5" t="s">
         <v>9</v>
       </c>
-      <c r="C3" t="s">
+      <c r="C5" t="s">
         <v>9</v>
       </c>
-      <c r="D3" t="s">
+      <c r="D5" t="s">
         <v>15</v>
       </c>
-      <c r="F3">
+      <c r="E5">
         <v>5</v>
       </c>
-      <c r="G3">
-        <v>0.8</v>
-      </c>
-      <c r="H3">
-        <v>1</v>
-      </c>
-      <c r="I3">
+      <c r="F5">
+        <v>1</v>
+      </c>
+      <c r="G5">
+        <v>1</v>
+      </c>
+      <c r="H5">
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A4">
-        <v>10004</v>
-      </c>
-      <c r="B4" t="s">
+    <row r="6" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A6">
+        <v>10005</v>
+      </c>
+      <c r="B6" t="s">
         <v>10</v>
       </c>
-      <c r="C4" t="s">
+      <c r="C6" t="s">
         <v>10</v>
       </c>
-      <c r="D4" t="s">
+      <c r="D6" t="s">
         <v>16</v>
       </c>
-      <c r="F4">
+      <c r="E6">
         <v>5</v>
       </c>
-      <c r="G4">
-        <v>1</v>
-      </c>
-      <c r="H4">
-        <v>1</v>
-      </c>
-      <c r="I4">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A5">
-        <v>10005</v>
-      </c>
-      <c r="B5" t="s">
-        <v>11</v>
-      </c>
-      <c r="C5" t="s">
-        <v>11</v>
-      </c>
-      <c r="D5" t="s">
-        <v>17</v>
-      </c>
-      <c r="F5">
-        <v>5</v>
-      </c>
-      <c r="G5">
-        <v>1</v>
-      </c>
-      <c r="H5">
-        <v>1</v>
-      </c>
-      <c r="I5">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A6">
-        <v>10006</v>
-      </c>
-      <c r="B6" t="s">
-        <v>12</v>
-      </c>
-      <c r="C6" t="s">
-        <v>12</v>
-      </c>
-      <c r="D6" t="s">
-        <v>18</v>
-      </c>
       <c r="F6">
-        <v>5</v>
+        <v>0.7</v>
       </c>
       <c r="G6">
-        <v>0.7</v>
+        <v>1</v>
       </c>
       <c r="H6">
-        <v>1</v>
-      </c>
-      <c r="I6">
         <v>1</v>
       </c>
     </row>

</xml_diff>

<commit_message>
[Update] UT 전 오류 개선
</commit_message>
<xml_diff>
--- a/Assets/Resources/Excels/MonsterSheets.xlsx
+++ b/Assets/Resources/Excels/MonsterSheets.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Project\In_You\Assets\Resources\Excels\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8E4AC8F3-45AC-4165-9D88-A144BDC8E22C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{69BDC178-6FBD-4C7F-B886-2787A94EF185}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{370970DB-CFD6-4742-B8DB-B40C1E5D66D6}"/>
   </bookViews>
@@ -537,10 +537,10 @@
         <v>1.1000000000000001</v>
       </c>
       <c r="G2">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="H2">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="I2">
         <v>10001</v>
@@ -566,10 +566,10 @@
         <v>0.8</v>
       </c>
       <c r="G3">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="H3">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="I3">
         <v>10002</v>
@@ -595,10 +595,10 @@
         <v>1</v>
       </c>
       <c r="G4">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="H4">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="I4">
         <v>10003</v>
@@ -624,10 +624,10 @@
         <v>1</v>
       </c>
       <c r="G5">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="H5">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="I5">
         <v>10004</v>
@@ -653,10 +653,10 @@
         <v>0.7</v>
       </c>
       <c r="G6">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="H6">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="I6">
         <v>10005</v>

</xml_diff>

<commit_message>
[Fix] Monster관련 오류 수정
</commit_message>
<xml_diff>
--- a/Assets/Resources/Excels/MonsterSheets.xlsx
+++ b/Assets/Resources/Excels/MonsterSheets.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Project\In_You\Assets\Resources\Excels\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{69BDC178-6FBD-4C7F-B886-2787A94EF185}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6E2D185F-8C49-4DA1-8CCD-AA178652C087}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{370970DB-CFD6-4742-B8DB-B40C1E5D66D6}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="19">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="20">
   <si>
     <t>displayTitle</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -84,27 +84,35 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>/Prefabs/Monster/Raven</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>/Prefabs/Monster/Spider</t>
-  </si>
-  <si>
-    <t>/Prefabs/Monster/RedZombie</t>
-  </si>
-  <si>
-    <t>/Prefabs/Monster/PurpleZombie</t>
-  </si>
-  <si>
-    <t>/Prefabs/Monster/CrawlZombie</t>
-  </si>
-  <si>
     <t>id</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
     <t>monsterID</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>attackDistance</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Monster/Raven</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Monster/Spider</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Monster/RedZombie</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Monster/PurpleZombie</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Monster/CrawlZombie</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -469,7 +477,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{02DBBB59-976D-468B-AEDF-09065DDEF90E}">
-  <dimension ref="A1:I6"/>
+  <dimension ref="A1:J6"/>
   <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="10.25" bestFit="1" customWidth="1"/>
@@ -488,9 +496,9 @@
     <col min="14" max="14" width="8.75" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
-        <v>17</v>
+        <v>12</v>
       </c>
       <c r="B1" t="s">
         <v>0</v>
@@ -514,10 +522,13 @@
         <v>5</v>
       </c>
       <c r="I1" t="s">
-        <v>18</v>
+        <v>14</v>
+      </c>
+      <c r="J1" t="s">
+        <v>13</v>
       </c>
     </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A2">
         <v>10001</v>
       </c>
@@ -528,7 +539,7 @@
         <v>11</v>
       </c>
       <c r="D2" t="s">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="E2">
         <v>5</v>
@@ -537,16 +548,19 @@
         <v>1.1000000000000001</v>
       </c>
       <c r="G2">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="H2">
         <v>10</v>
       </c>
       <c r="I2">
+        <v>1.5</v>
+      </c>
+      <c r="J2">
         <v>10001</v>
       </c>
     </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A3">
         <v>10002</v>
       </c>
@@ -557,7 +571,7 @@
         <v>7</v>
       </c>
       <c r="D3" t="s">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="E3">
         <v>5</v>
@@ -566,16 +580,19 @@
         <v>0.8</v>
       </c>
       <c r="G3">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="H3">
         <v>10</v>
       </c>
       <c r="I3">
+        <v>1.5</v>
+      </c>
+      <c r="J3">
         <v>10002</v>
       </c>
     </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A4">
         <v>10003</v>
       </c>
@@ -586,7 +603,7 @@
         <v>8</v>
       </c>
       <c r="D4" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="E4">
         <v>5</v>
@@ -595,16 +612,19 @@
         <v>1</v>
       </c>
       <c r="G4">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="H4">
         <v>10</v>
       </c>
       <c r="I4">
+        <v>1.5</v>
+      </c>
+      <c r="J4">
         <v>10003</v>
       </c>
     </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A5">
         <v>10004</v>
       </c>
@@ -615,7 +635,7 @@
         <v>9</v>
       </c>
       <c r="D5" t="s">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="E5">
         <v>5</v>
@@ -624,16 +644,19 @@
         <v>1</v>
       </c>
       <c r="G5">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="H5">
         <v>10</v>
       </c>
       <c r="I5">
+        <v>1.5</v>
+      </c>
+      <c r="J5">
         <v>10004</v>
       </c>
     </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A6">
         <v>10005</v>
       </c>
@@ -644,7 +667,7 @@
         <v>10</v>
       </c>
       <c r="D6" t="s">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="E6">
         <v>5</v>
@@ -653,12 +676,15 @@
         <v>0.7</v>
       </c>
       <c r="G6">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="H6">
         <v>10</v>
       </c>
       <c r="I6">
+        <v>1.5</v>
+      </c>
+      <c r="J6">
         <v>10005</v>
       </c>
     </row>

</xml_diff>